<commit_message>
Add 'Action Items Mapping' sheet — reverse view: each docx item → KPI(s)
Sheet1 = KPI-first (each KPI shows which action item it addresses).
NEW Sheet2 = Item-first (each of the 15 docx items shows which KPI(s)
address it and which panel(s) implement it).

Columns on the new sheet:
  A  Item #                  (1–15)
  B  Action Item (from docx) (full description)
  C  # KPIs                  (count of KPIs addressing this item)
  D  KPI(s) Addressing It    (from Sheet1)
  E  Panel(s) in v2          (specific enhanced-dashboard panel names)
  F  Status                  (Achieved / Achieved (removed) / No change needed)

All 15 items covered; counts range from 1 to 4 KPIs per item.

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017VYgevi2qMhpc8f2EWn1mG
</commit_message>
<xml_diff>
--- a/MIM_KPI_updated.xlsx
+++ b/MIM_KPI_updated.xlsx
@@ -7,6 +7,7 @@
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Action Items Mapping" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -80,7 +81,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
@@ -99,6 +100,12 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1746,4 +1753,478 @@
     <firstFooter/>
   </headerFooter>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F16"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="44" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="3" max="3"/>
+    <col width="42" customWidth="1" min="4" max="4"/>
+    <col width="42" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="8" t="inlineStr">
+        <is>
+          <t>Item #</t>
+        </is>
+      </c>
+      <c r="B1" s="8" t="inlineStr">
+        <is>
+          <t>Action Item (from docx)</t>
+        </is>
+      </c>
+      <c r="C1" s="8" t="inlineStr">
+        <is>
+          <t># KPIs</t>
+        </is>
+      </c>
+      <c r="D1" s="8" t="inlineStr">
+        <is>
+          <t>KPI(s) Addressing It</t>
+        </is>
+      </c>
+      <c r="E1" s="8" t="inlineStr">
+        <is>
+          <t>Enhanced Dashboard v2 Panel(s)</t>
+        </is>
+      </c>
+      <c r="F1" s="8" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="80" customHeight="1">
+      <c r="A2" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="9" t="inlineStr">
+        <is>
+          <t>Active P1/P2 Panel — enhance to identify incidents requiring action; provide visibility into tickets pending assignment / investigation / resolution; replace CI Number with CI Name; add Support Group and Status columns</t>
+        </is>
+      </c>
+      <c r="C2" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="D2" s="9" t="inlineStr">
+        <is>
+          <t># Active Major Incidents; Open Incident Ageing (merged into #1); Active P1/P2 — Pending Action Table</t>
+        </is>
+      </c>
+      <c r="E2" s="9" t="inlineStr">
+        <is>
+          <t>'Active Major Incidents' metric tile + 'Active P1/P2 — Pending Action' datatable</t>
+        </is>
+      </c>
+      <c r="F2" s="8" t="inlineStr">
+        <is>
+          <t>Achieved</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="80" customHeight="1">
+      <c r="A3" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="9" t="inlineStr">
+        <is>
+          <t>Resolved/Opened Panel — review and clarify calculation logic; confirm whether metric is based on Open P1/P2 only or all P1/P2 within reporting period; update widget definition and tooltip</t>
+        </is>
+      </c>
+      <c r="C3" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="D3" s="9" t="inlineStr">
+        <is>
+          <t>Action Closure Rate; Closure Rate %</t>
+        </is>
+      </c>
+      <c r="E3" s="9" t="inlineStr">
+        <is>
+          <t>'Closure Rate (P1+P2)' metric tile — denominator = all P1+P2 opened in window; numerator = COUNT(resolved_at)</t>
+        </is>
+      </c>
+      <c r="F3" s="8" t="inlineStr">
+        <is>
+          <t>Achieved</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="80" customHeight="1">
+      <c r="A4" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="9" t="inlineStr">
+        <is>
+          <t>Drill-Down Capability — add drill-down to all widgets containing line graphs; users should click a data point and view underlying incident records</t>
+        </is>
+      </c>
+      <c r="C4" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="D4" s="9" t="inlineStr">
+        <is>
+          <t>Incident Volume Over Time; MTTR Trend by Priority (P1 vs P2)</t>
+        </is>
+      </c>
+      <c r="E4" s="9" t="inlineStr">
+        <is>
+          <t>'Incident Volume Over Time (by Priority)' and 'MTTR Trend (Median per day, split by P1 &amp; P2)' — Kibana default click-to-filter behaviour applies to both</t>
+        </is>
+      </c>
+      <c r="F4" s="8" t="inlineStr">
+        <is>
+          <t>Achieved</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="80" customHeight="1">
+      <c r="A5" s="8" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="9" t="inlineStr">
+        <is>
+          <t>MTTR Trend (Median P1+P2 Per Day) — implement separate MTTR trends for P1 and P2 (or drill-down showing MTTR tickets)</t>
+        </is>
+      </c>
+      <c r="C5" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="D5" s="9" t="inlineStr">
+        <is>
+          <t>MTTR; MTTR Trend by Priority (P1 vs P2)</t>
+        </is>
+      </c>
+      <c r="E5" s="9" t="inlineStr">
+        <is>
+          <t>'MTTR Trend (Median per day, split by P1 &amp; P2)' line chart — multi-series</t>
+        </is>
+      </c>
+      <c r="F5" s="8" t="inlineStr">
+        <is>
+          <t>Achieved</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="80" customHeight="1">
+      <c r="A6" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="9" t="inlineStr">
+        <is>
+          <t>Incidents by CI / Support Team — restrict data to P1 and P2 incidents only</t>
+        </is>
+      </c>
+      <c r="C6" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="D6" s="9" t="inlineStr">
+        <is>
+          <t>Incidents by Service/Team</t>
+        </is>
+      </c>
+      <c r="E6" s="9" t="inlineStr">
+        <is>
+          <t>'Incidents by CI / Support Team (P1+P2 Only)' datatable — added WHERE priority IN (1,2), dropped P3 column</t>
+        </is>
+      </c>
+      <c r="F6" s="8" t="inlineStr">
+        <is>
+          <t>Achieved</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="80" customHeight="1">
+      <c r="A7" s="8" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="9" t="inlineStr">
+        <is>
+          <t>Percentage of CIs with Major Incidents — convert to drill-down enabled widget; add detailed table showing CIs associated with more than one major incident</t>
+        </is>
+      </c>
+      <c r="C7" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="D7" s="9" t="inlineStr">
+        <is>
+          <t>Recurrence Rate</t>
+        </is>
+      </c>
+      <c r="E7" s="9" t="inlineStr">
+        <is>
+          <t>'Recurrence Rate (P1+P2)' metric tile + 'Repeat-Offender CIs (&gt;1 P1/P2 Incident)' pie (the drill-down detail)</t>
+        </is>
+      </c>
+      <c r="F7" s="8" t="inlineStr">
+        <is>
+          <t>Achieved</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="80" customHeight="1">
+      <c r="A8" s="8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="9" t="inlineStr">
+        <is>
+          <t>Repeat Offenders — convert the existing table into a pie chart</t>
+        </is>
+      </c>
+      <c r="C8" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="D8" s="9" t="inlineStr">
+        <is>
+          <t>Recurrence Rate</t>
+        </is>
+      </c>
+      <c r="E8" s="9" t="inlineStr">
+        <is>
+          <t>'Repeat-Offender CIs (&gt;1 P1/P2 Incident)' pie chart — converted from datatable</t>
+        </is>
+      </c>
+      <c r="F8" s="8" t="inlineStr">
+        <is>
+          <t>Achieved</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="80" customHeight="1">
+      <c r="A9" s="8" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="9" t="inlineStr">
+        <is>
+          <t>Detection Source — convert the existing table into a pie chart</t>
+        </is>
+      </c>
+      <c r="C9" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="D9" s="9" t="inlineStr">
+        <is>
+          <t>Detection Source Ratio</t>
+        </is>
+      </c>
+      <c r="E9" s="9" t="inlineStr">
+        <is>
+          <t>'Detection Source (All Incidents)' pie chart — converted from datatable</t>
+        </is>
+      </c>
+      <c r="F9" s="8" t="inlineStr">
+        <is>
+          <t>Achieved</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="80" customHeight="1">
+      <c r="A10" s="8" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="9" t="inlineStr">
+        <is>
+          <t>Alert vs Auto-Generated Incidents — add new widget between Detection Source and Top Affected CIs showing alert-generated and auto-generated incidents; validate source field</t>
+        </is>
+      </c>
+      <c r="C10" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="D10" s="9" t="inlineStr">
+        <is>
+          <t>Alert vs Auto-Generated Incidents</t>
+        </is>
+      </c>
+      <c r="E10" s="9" t="inlineStr">
+        <is>
+          <t>'Alert vs Auto-Generated Incidents' pie chart — uses existing contact_type values 'alert' and 'auto_generated' (both confirmed present in the index; no new field required)</t>
+        </is>
+      </c>
+      <c r="F10" s="8" t="inlineStr">
+        <is>
+          <t>Achieved</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="80" customHeight="1">
+      <c r="A11" s="8" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="9" t="inlineStr">
+        <is>
+          <t>Open Incidents — no changes required</t>
+        </is>
+      </c>
+      <c r="C11" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="D11" s="9" t="inlineStr">
+        <is>
+          <t>Open Incident Ageing</t>
+        </is>
+      </c>
+      <c r="E11" s="9" t="inlineStr">
+        <is>
+          <t>'Active P1/P2 — Pending Action' datatable (also serves this view)</t>
+        </is>
+      </c>
+      <c r="F11" s="8" t="inlineStr">
+        <is>
+          <t>No change needed</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="80" customHeight="1">
+      <c r="A12" s="8" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="9" t="inlineStr">
+        <is>
+          <t>Aging Analysis — no changes required</t>
+        </is>
+      </c>
+      <c r="C12" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="D12" s="9" t="inlineStr">
+        <is>
+          <t>Open Incident Ageing</t>
+        </is>
+      </c>
+      <c r="E12" s="9" t="inlineStr">
+        <is>
+          <t>'Active P1/P2 — Pending Action' datatable — merged with Aging Analysis into a single actionable table per item #1</t>
+        </is>
+      </c>
+      <c r="F12" s="8" t="inlineStr">
+        <is>
+          <t>No change needed</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="80" customHeight="1">
+      <c r="A13" s="8" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="9" t="inlineStr">
+        <is>
+          <t>Business Service Impact (P1+P2) — remove the Business Service Impact panel</t>
+        </is>
+      </c>
+      <c r="C13" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="D13" s="9" t="inlineStr">
+        <is>
+          <t>Business Service Impact</t>
+        </is>
+      </c>
+      <c r="E13" s="9" t="inlineStr">
+        <is>
+          <t>REMOVED from the dashboard</t>
+        </is>
+      </c>
+      <c r="F13" s="8" t="inlineStr">
+        <is>
+          <t>Achieved (removed)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="80" customHeight="1">
+      <c r="A14" s="8" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="9" t="inlineStr">
+        <is>
+          <t>Assignment Group Load (P1+P2 Incidents) — change visualization from a table to a pie chart</t>
+        </is>
+      </c>
+      <c r="C14" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="D14" s="9" t="inlineStr">
+        <is>
+          <t>Assignment Group Load</t>
+        </is>
+      </c>
+      <c r="E14" s="9" t="inlineStr">
+        <is>
+          <t>'Assignment Group Load (P1+P2)' pie chart — converted from datatable</t>
+        </is>
+      </c>
+      <c r="F14" s="8" t="inlineStr">
+        <is>
+          <t>Achieved</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="80" customHeight="1">
+      <c r="A15" s="8" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="9" t="inlineStr">
+        <is>
+          <t>SLA Monitoring for Open P1/P2 Tickets — add SLA-focused widgets: SLA Breached, SLA At Risk / Will Breach Soon, SLA Status Overview (Within / Approaching / Breached); enable drill-down on all SLA widgets</t>
+        </is>
+      </c>
+      <c r="C15" s="8" t="n">
+        <v>4</v>
+      </c>
+      <c r="D15" s="9" t="inlineStr">
+        <is>
+          <t>SLO Impact Rate (substitute); SLA Breached (Open P1/P2); SLA At Risk (Approaching Breach); SLA Within Target</t>
+        </is>
+      </c>
+      <c r="E15" s="9" t="inlineStr">
+        <is>
+          <t>'SLA Breached (Open P1/P2)' + 'SLA At Risk (&gt;=80% of target)' + 'SLA Within Target' metric tiles. SLA targets are ITIL defaults (P1=4h, P2=8h); adjust the CASE expression to match the actual SLA agreement</t>
+        </is>
+      </c>
+      <c r="F15" s="8" t="inlineStr">
+        <is>
+          <t>Achieved</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="80" customHeight="1">
+      <c r="A16" s="8" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" s="9" t="inlineStr">
+        <is>
+          <t>SLA Breach Detail View — clicking any SLA-related widget should open a detailed table showing: Incident #, Priority, State, Assigned Group, CI Name, Ticket Age, SLA Target, SLA Status, Time Remaining / Time Overdue</t>
+        </is>
+      </c>
+      <c r="C16" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="D16" s="9" t="inlineStr">
+        <is>
+          <t>SLO Impact Rate (substitute); SLA Breach Detail Table</t>
+        </is>
+      </c>
+      <c r="E16" s="9" t="inlineStr">
+        <is>
+          <t>'SLA Breach Detail — Open P1/P2 Incidents' datatable with every requested column. Kibana default click-to-filter satisfies the 'clicking any SLA widget' request</t>
+        </is>
+      </c>
+      <c r="F16" s="8" t="inlineStr">
+        <is>
+          <t>Achieved</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>